<commit_message>
Switch to the new October workbook format
- template/template.xlsx rebuilt from the owner's final sale Oct-2025
  workbook (now kept as template/sample sale Oct-2025.xlsx; the Nov-2025
  sample is removed). All its formulas are kept: qty from rows 13-15,
  Paytm/PhonePe 60/40 petrol/diesel split, ICICI and HP litres.
- Cash qty Q4:Q6 is now filled as sale qty - Paytm share - ICICI -
  PhonePe share - HP card - udhar qty (matches the owner's file on all
  31 days). K17 ICICI copy and the Sheet1 register are no longer written.
- October readings for days 19, 22 and 24 updated to the owner's
  corrected values; the rebuilt October workbook now matches the owner's
  file cell for cell (apart from scratch notes).
- Tests for the new format (33 passing); README updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QV4oMj4LEVDz3Zb3PjxM1z
</commit_message>
<xml_diff>
--- a/template/template.xlsx
+++ b/template/template.xlsx
@@ -3,11 +3,10 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" tabRatio="600" firstSheet="19" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9060" tabRatio="600" firstSheet="23" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="TEMPLATE" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -16,11 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.00_ "/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,12 +78,6 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -99,7 +93,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="27">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -177,42 +171,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
-      <right/>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
       <top style="thin">
         <color auto="1"/>
       </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -233,7 +201,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color theme="4" tint="0.3998535111545152"/>
+        <color theme="4" tint="0.3998229926450392"/>
       </bottom>
       <diagonal/>
     </border>
@@ -339,13 +307,52 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
         <color auto="1"/>
       </left>
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -359,6 +366,17 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
       <top style="double">
@@ -369,50 +387,13 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right style="thick">
         <color auto="1"/>
       </right>
       <top style="thin">
         <color auto="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color auto="1"/>
-      </left>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -420,17 +401,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -455,7 +430,7 @@
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -477,22 +452,22 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -508,87 +483,90 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="43" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -936,26 +914,26 @@
   <dimension ref="A1:X50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
-    <col width="13.109375" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13.109375" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10.109375" customWidth="1" min="7" max="7"/>
-    <col width="10.6640625" customWidth="1" min="8" max="8"/>
-    <col width="9.5546875" customWidth="1" min="9" max="9"/>
-    <col width="10.6640625" customWidth="1" min="10" max="14"/>
-    <col width="13.44140625" customWidth="1" min="15" max="15"/>
-    <col width="11.88671875" customWidth="1" min="16" max="16"/>
-    <col width="10.6640625" customWidth="1" min="18" max="18"/>
-    <col width="9.5546875" customWidth="1" min="19" max="19"/>
-    <col width="10.6640625" customWidth="1" min="20" max="20"/>
-    <col width="9.6640625" customWidth="1" min="21" max="21"/>
-    <col width="12.5546875" customWidth="1" min="23" max="23"/>
-    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="13.109375" customWidth="1" style="69" min="1" max="1"/>
+    <col width="12" customWidth="1" style="69" min="2" max="2"/>
+    <col width="12" customWidth="1" style="69" min="4" max="4"/>
+    <col width="13.109375" customWidth="1" style="69" min="5" max="5"/>
+    <col width="14" customWidth="1" style="69" min="6" max="6"/>
+    <col width="10.109375" customWidth="1" style="69" min="7" max="7"/>
+    <col width="10.6640625" customWidth="1" style="69" min="8" max="8"/>
+    <col width="9.5546875" customWidth="1" style="69" min="9" max="9"/>
+    <col width="10.6640625" customWidth="1" style="69" min="10" max="14"/>
+    <col width="13.44140625" customWidth="1" style="69" min="15" max="15"/>
+    <col width="11.88671875" customWidth="1" style="69" min="16" max="16"/>
+    <col width="10.6640625" customWidth="1" style="69" min="18" max="18"/>
+    <col width="9.5546875" customWidth="1" style="69" min="19" max="19"/>
+    <col width="10.6640625" customWidth="1" style="69" min="20" max="20"/>
+    <col width="9.6640625" customWidth="1" style="69" min="21" max="21"/>
+    <col width="12.5546875" customWidth="1" style="69" min="23" max="23"/>
+    <col width="12" customWidth="1" style="69" min="24" max="24"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.6" customHeight="1">
+    <row r="1" ht="18.6" customHeight="1" s="69">
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
@@ -977,251 +955,251 @@
       <c r="T1" s="1" t="n"/>
       <c r="U1" s="1" t="n"/>
     </row>
-    <row r="2" ht="18.6" customHeight="1">
-      <c r="A2" s="64" t="inlineStr">
+    <row r="2" ht="18.6" customHeight="1" s="69">
+      <c r="A2" s="47" t="inlineStr">
         <is>
           <t>Particular</t>
         </is>
       </c>
-      <c r="B2" s="64" t="inlineStr">
+      <c r="B2" s="47" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="C2" s="64" t="inlineStr">
+      <c r="C2" s="47" t="inlineStr">
         <is>
           <t>Rate</t>
         </is>
       </c>
-      <c r="D2" s="65" t="inlineStr">
+      <c r="D2" s="50" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="E2" s="60" t="inlineStr">
+      <c r="E2" s="56" t="inlineStr">
         <is>
           <t>Pos SBI</t>
         </is>
       </c>
-      <c r="F2" s="66" t="n"/>
-      <c r="G2" s="60" t="inlineStr">
+      <c r="F2" s="57" t="n"/>
+      <c r="G2" s="56" t="inlineStr">
         <is>
           <t>Paytm</t>
         </is>
       </c>
-      <c r="H2" s="66" t="n"/>
-      <c r="I2" s="60" t="inlineStr">
+      <c r="H2" s="57" t="n"/>
+      <c r="I2" s="56" t="inlineStr">
         <is>
           <t>HP Card</t>
         </is>
       </c>
-      <c r="J2" s="66" t="n"/>
-      <c r="K2" s="60" t="inlineStr">
+      <c r="J2" s="57" t="n"/>
+      <c r="K2" s="56" t="inlineStr">
         <is>
           <t>ICICI</t>
         </is>
       </c>
-      <c r="L2" s="66" t="n"/>
-      <c r="M2" s="60" t="inlineStr">
+      <c r="L2" s="57" t="n"/>
+      <c r="M2" s="56" t="inlineStr">
         <is>
           <t>phone pe</t>
         </is>
       </c>
-      <c r="N2" s="66" t="n"/>
-      <c r="O2" s="67" t="inlineStr">
+      <c r="N2" s="57" t="n"/>
+      <c r="O2" s="54" t="inlineStr">
         <is>
           <t>mobiquick</t>
         </is>
       </c>
-      <c r="P2" s="68" t="n"/>
-      <c r="Q2" s="60" t="inlineStr">
+      <c r="P2" s="55" t="n"/>
+      <c r="Q2" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">CASH </t>
         </is>
       </c>
-      <c r="R2" s="66" t="n"/>
-      <c r="S2" s="60" t="inlineStr">
+      <c r="R2" s="57" t="n"/>
+      <c r="S2" s="56" t="inlineStr">
         <is>
           <t>Credit</t>
         </is>
       </c>
-      <c r="T2" s="66" t="n"/>
-      <c r="U2" s="69" t="inlineStr">
+      <c r="T2" s="57" t="n"/>
+      <c r="U2" s="45" t="inlineStr">
         <is>
           <t>Qty Diffrence</t>
         </is>
       </c>
-      <c r="W2" s="4" t="n"/>
-      <c r="X2" s="4" t="n"/>
-    </row>
-    <row r="3" ht="18.6" customHeight="1">
-      <c r="A3" s="70" t="n"/>
-      <c r="B3" s="70" t="n"/>
-      <c r="C3" s="70" t="n"/>
-      <c r="D3" s="71" t="n"/>
-      <c r="E3" s="60" t="inlineStr">
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="18.6" customHeight="1" s="69">
+      <c r="A3" s="46" t="n"/>
+      <c r="B3" s="46" t="n"/>
+      <c r="C3" s="46" t="n"/>
+      <c r="D3" s="51" t="n"/>
+      <c r="E3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="F3" s="61" t="inlineStr">
+      <c r="F3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="G3" s="60" t="inlineStr">
+      <c r="G3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="H3" s="61" t="inlineStr">
+      <c r="H3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="I3" s="60" t="inlineStr">
+      <c r="I3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="J3" s="61" t="inlineStr">
+      <c r="J3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="K3" s="60" t="inlineStr">
+      <c r="K3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="L3" s="61" t="inlineStr">
+      <c r="L3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="M3" s="60" t="inlineStr">
+      <c r="M3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="N3" s="61" t="inlineStr">
+      <c r="N3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="O3" s="60" t="inlineStr">
+      <c r="O3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="P3" s="61" t="inlineStr">
+      <c r="P3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="Q3" s="60" t="inlineStr">
+      <c r="Q3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="R3" s="61" t="inlineStr">
+      <c r="R3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="S3" s="60" t="inlineStr">
+      <c r="S3" s="56" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="T3" s="61" t="inlineStr">
+      <c r="T3" s="41" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="U3" s="70" t="n"/>
-      <c r="W3" s="4" t="inlineStr">
+      <c r="U3" s="46" t="n"/>
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="X3" s="4">
+      <c r="X3" s="2">
         <f>+SUMIFS(C15:C25,B15:B25,W3)</f>
         <v/>
       </c>
     </row>
-    <row r="4" customFormat="1" s="4">
-      <c r="A4" s="5" t="inlineStr">
+    <row r="4" customFormat="1" s="2">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Petrol</t>
         </is>
       </c>
-      <c r="B4" s="14">
-        <f>H16</f>
-        <v/>
-      </c>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="7">
+      <c r="B4" s="12">
+        <f>+(H13+H14+H15)/$C$4</f>
+        <v/>
+      </c>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="5">
         <f>B4*C4</f>
         <v/>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="7">
         <f>+E4*C4</f>
         <v/>
       </c>
-      <c r="G4" s="8">
-        <f>+K20</f>
-        <v/>
-      </c>
-      <c r="H4" s="9">
+      <c r="G4" s="9">
+        <f>+(H8*60%)/$C$4</f>
+        <v/>
+      </c>
+      <c r="H4" s="7">
         <f>+G4*C4</f>
         <v/>
       </c>
-      <c r="I4" s="8">
+      <c r="I4" s="6">
         <f>J4/C4</f>
         <v/>
       </c>
-      <c r="J4" s="9" t="n">
+      <c r="J4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="10">
-        <f>+M17</f>
-        <v/>
-      </c>
-      <c r="L4" s="9">
+      <c r="K4" s="8">
+        <f>+L8/$C$4</f>
+        <v/>
+      </c>
+      <c r="L4" s="7">
         <f>+K4*C4</f>
         <v/>
       </c>
-      <c r="M4" s="11">
-        <f>+M15</f>
-        <v/>
-      </c>
-      <c r="N4" s="9">
+      <c r="M4" s="9">
+        <f>+(N8*60%)/$C$4</f>
+        <v/>
+      </c>
+      <c r="N4" s="7">
         <f>+M4*C4</f>
         <v/>
       </c>
-      <c r="O4" s="11" t="n"/>
-      <c r="P4" s="9">
+      <c r="O4" s="9" t="n"/>
+      <c r="P4" s="7">
         <f>+O4*C4</f>
         <v/>
       </c>
-      <c r="Q4" s="8" t="n"/>
-      <c r="R4" s="9">
+      <c r="Q4" s="6" t="n"/>
+      <c r="R4" s="7">
         <f>+Q4*C4</f>
         <v/>
       </c>
-      <c r="S4" s="12">
+      <c r="S4" s="10">
         <f>+X4</f>
         <v/>
       </c>
-      <c r="T4" s="9">
+      <c r="T4" s="7">
         <f>+S4*C4</f>
         <v/>
       </c>
-      <c r="U4" s="13">
+      <c r="U4" s="11">
         <f>+B4-E4-G4-Q4-S4-K4-I4-M4-O4</f>
         <v/>
       </c>
@@ -1230,86 +1208,86 @@
           <t>petrol</t>
         </is>
       </c>
-      <c r="X4" s="4">
+      <c r="X4" s="2">
         <f>+SUMIFS(C15:C26,B15:B26,W4)</f>
         <v/>
       </c>
     </row>
-    <row r="5" customFormat="1" s="4">
-      <c r="A5" s="5" t="inlineStr">
+    <row r="5" customFormat="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Diesal</t>
         </is>
       </c>
-      <c r="B5" s="14">
-        <f>I16</f>
-        <v/>
-      </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="7">
+      <c r="B5" s="12">
+        <f>+(I13+I14+I15)/$C$5</f>
+        <v/>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="5">
         <f>B5*C5</f>
         <v/>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <f>+E5*C5</f>
         <v/>
       </c>
-      <c r="G5" s="8">
-        <f>+M16</f>
-        <v/>
-      </c>
-      <c r="H5" s="9">
+      <c r="G5" s="6">
+        <f>+(H8*40%)/$C$5</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
         <f>+G5*C5</f>
         <v/>
       </c>
-      <c r="I5" s="8">
+      <c r="I5" s="6">
         <f>+J8/C5</f>
         <v/>
       </c>
-      <c r="J5" s="9">
+      <c r="J5" s="7">
         <f>+I5*C5</f>
         <v/>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="9">
+      <c r="L5" s="7">
         <f>+K5*C5</f>
         <v/>
       </c>
-      <c r="M5" s="11">
-        <f>+M19</f>
-        <v/>
-      </c>
-      <c r="N5" s="9">
+      <c r="M5" s="6">
+        <f>+(N8*40%)/$C$5</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
         <f>+M5*C5</f>
         <v/>
       </c>
-      <c r="O5" s="11">
+      <c r="O5" s="9">
         <f>+P8/C5</f>
         <v/>
       </c>
-      <c r="P5" s="9">
+      <c r="P5" s="7">
         <f>+O5*C5</f>
         <v/>
       </c>
-      <c r="Q5" s="8" t="n"/>
-      <c r="R5" s="9">
+      <c r="Q5" s="6" t="n"/>
+      <c r="R5" s="7">
         <f>+Q5*C5</f>
         <v/>
       </c>
-      <c r="S5" s="12">
+      <c r="S5" s="10">
         <f>+X3</f>
         <v/>
       </c>
-      <c r="T5" s="9">
+      <c r="T5" s="7">
         <f>+S5*C5</f>
         <v/>
       </c>
-      <c r="U5" s="13">
+      <c r="U5" s="11">
         <f>+B5-E5-G5-Q5-S5-K5-I5-M5-O5</f>
         <v/>
       </c>
@@ -1318,780 +1296,610 @@
           <t>Petrol Power</t>
         </is>
       </c>
-      <c r="X5" s="4">
+      <c r="X5" s="2">
         <f>+SUMIFS(C17:C27,B17:B27,W5)</f>
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="1" s="4">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" customFormat="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Petrol Power</t>
         </is>
       </c>
-      <c r="B6" s="14">
-        <f>J16</f>
-        <v/>
-      </c>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="7">
+      <c r="B6" s="12">
+        <f>+(J13+J14+J15)/$C$6</f>
+        <v/>
+      </c>
+      <c r="C6" s="4" t="n"/>
+      <c r="D6" s="5">
         <f>B6*C6</f>
         <v/>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="7">
         <f>+E6*C6</f>
         <v/>
       </c>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="9">
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="7">
         <f>+G6*C6</f>
         <v/>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="9">
+      <c r="J6" s="7">
         <f>+I6*C6</f>
         <v/>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="L6" s="9">
+      <c r="L6" s="7">
         <f>+K6*C6</f>
         <v/>
       </c>
-      <c r="M6" s="11" t="n">
+      <c r="M6" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="N6" s="9">
+      <c r="N6" s="7">
         <f>+M6*C6</f>
         <v/>
       </c>
-      <c r="O6" s="11" t="n"/>
-      <c r="P6" s="9">
+      <c r="O6" s="9" t="n"/>
+      <c r="P6" s="7">
         <f>+O6*C6</f>
         <v/>
       </c>
-      <c r="Q6" s="8" t="n"/>
-      <c r="R6" s="9">
+      <c r="Q6" s="6" t="n"/>
+      <c r="R6" s="7">
         <f>+Q6*C6</f>
         <v/>
       </c>
-      <c r="S6" s="12">
+      <c r="S6" s="10">
         <f>+X5</f>
         <v/>
       </c>
-      <c r="T6" s="9">
+      <c r="T6" s="7">
         <f>+S6*C6</f>
         <v/>
       </c>
-      <c r="U6" s="13">
+      <c r="U6" s="11">
         <f>+B6-E6-G6-Q6-S6-K6-I6-M6-O6</f>
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="1" s="4">
-      <c r="A7" s="5" t="n"/>
-      <c r="B7" s="46">
+    <row r="7" customFormat="1" s="2">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="38">
         <f>SUM(B4:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="15">
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="13">
         <f>SUM(D4:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="16">
+      <c r="E7" s="14">
         <f>SUM(E4:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="15">
         <f>SUM(F4:F6)</f>
         <v/>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="14">
         <f>SUM(G4:G6)</f>
         <v/>
       </c>
-      <c r="H7" s="17">
+      <c r="H7" s="15">
         <f>SUM(H4:H6)</f>
         <v/>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="14">
         <f>SUM(I4:I6)</f>
         <v/>
       </c>
-      <c r="J7" s="17">
+      <c r="J7" s="15">
         <f>SUM(J4:J6)</f>
         <v/>
       </c>
-      <c r="K7" s="16">
+      <c r="K7" s="14">
         <f>SUM(K4:K6)</f>
         <v/>
       </c>
-      <c r="L7" s="17">
+      <c r="L7" s="15">
         <f>SUM(L4:L6)</f>
         <v/>
       </c>
-      <c r="M7" s="16">
+      <c r="M7" s="14">
         <f>SUM(M4:M6)</f>
         <v/>
       </c>
-      <c r="N7" s="17">
+      <c r="N7" s="15">
         <f>SUM(N4:N6)</f>
         <v/>
       </c>
-      <c r="O7" s="16">
+      <c r="O7" s="14">
         <f>SUM(O4:O6)</f>
         <v/>
       </c>
-      <c r="P7" s="17">
+      <c r="P7" s="15">
         <f>SUM(P4:P6)</f>
         <v/>
       </c>
-      <c r="Q7" s="16">
+      <c r="Q7" s="14">
         <f>SUM(Q4:Q6)</f>
         <v/>
       </c>
-      <c r="R7" s="17">
+      <c r="R7" s="15">
         <f>SUM(R4:R6)</f>
         <v/>
       </c>
-      <c r="S7" s="16">
+      <c r="S7" s="14">
         <f>SUM(S4:S6)</f>
         <v/>
       </c>
-      <c r="T7" s="17">
+      <c r="T7" s="15">
         <f>SUM(T4:T6)</f>
         <v/>
       </c>
-      <c r="U7" s="13">
+      <c r="U7" s="11">
         <f>+B7-E7-G7-Q7-S7-K7-I7-M7-O7</f>
         <v/>
       </c>
     </row>
-    <row r="8" ht="15" customFormat="1" customHeight="1" s="4" thickBot="1">
-      <c r="A8" s="55" t="inlineStr">
+    <row r="8" ht="15" customFormat="1" customHeight="1" s="2" thickBot="1">
+      <c r="A8" s="52" t="inlineStr">
         <is>
           <t>Actual Amount</t>
         </is>
       </c>
-      <c r="B8" s="72" t="n"/>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="19" t="n"/>
-      <c r="E8" s="20" t="n"/>
-      <c r="F8" s="21" t="n">
+      <c r="B8" s="53" t="n"/>
+      <c r="C8" s="16" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="18" t="n"/>
+      <c r="F8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="20" t="n"/>
-      <c r="H8" s="21" t="n"/>
-      <c r="I8" s="20" t="n"/>
-      <c r="J8" s="21" t="n"/>
-      <c r="K8" s="20" t="n"/>
-      <c r="L8" s="21" t="n"/>
-      <c r="M8" s="22" t="n"/>
-      <c r="N8" s="21" t="n"/>
-      <c r="O8" s="22" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="P8" s="21" t="n">
+      <c r="G8" s="18" t="n"/>
+      <c r="H8" s="19" t="n"/>
+      <c r="I8" s="18" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="18" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="20" t="n"/>
+      <c r="N8" s="19" t="n"/>
+      <c r="O8" s="20" t="inlineStr"/>
+      <c r="P8" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="20" t="n">
+      <c r="Q8" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="R8" s="21" t="n"/>
-      <c r="S8" s="20" t="n"/>
-      <c r="T8" s="21" t="n"/>
-      <c r="U8" s="19" t="n"/>
-    </row>
-    <row r="9" ht="15.6" customHeight="1" thickBot="1" thickTop="1">
-      <c r="A9" s="57" t="inlineStr">
+      <c r="R8" s="19" t="n"/>
+      <c r="S8" s="18" t="n"/>
+      <c r="T8" s="19" t="n"/>
+      <c r="U8" s="17" t="n"/>
+    </row>
+    <row r="9" ht="15.6" customHeight="1" s="69" thickBot="1" thickTop="1">
+      <c r="A9" s="48" t="inlineStr">
         <is>
           <t>Diffrence should be zero</t>
         </is>
       </c>
-      <c r="B9" s="73" t="n"/>
-      <c r="C9" s="73" t="n"/>
-      <c r="D9" s="23" t="n"/>
-      <c r="E9" s="23" t="n"/>
-      <c r="F9" s="24">
+      <c r="B9" s="49" t="n"/>
+      <c r="C9" s="49" t="n"/>
+      <c r="D9" s="21" t="n"/>
+      <c r="E9" s="21" t="n"/>
+      <c r="F9" s="22">
         <f>+F7-F8</f>
         <v/>
       </c>
-      <c r="G9" s="23" t="n"/>
-      <c r="H9" s="24">
+      <c r="G9" s="21" t="n"/>
+      <c r="H9" s="22">
         <f>+H7-H8</f>
         <v/>
       </c>
-      <c r="I9" s="23" t="n"/>
-      <c r="J9" s="24">
+      <c r="I9" s="21" t="n"/>
+      <c r="J9" s="22">
         <f>+J7-J8</f>
         <v/>
       </c>
-      <c r="K9" s="23" t="n"/>
-      <c r="L9" s="24">
+      <c r="K9" s="21" t="n"/>
+      <c r="L9" s="22">
         <f>+L7-L8</f>
         <v/>
       </c>
-      <c r="M9" s="24" t="n"/>
-      <c r="N9" s="24">
+      <c r="M9" s="22" t="n"/>
+      <c r="N9" s="22">
         <f>+N7-N8</f>
         <v/>
       </c>
-      <c r="O9" s="24" t="n"/>
-      <c r="P9" s="24">
+      <c r="O9" s="22" t="n"/>
+      <c r="P9" s="22">
         <f>+P7-P8</f>
         <v/>
       </c>
-      <c r="Q9" s="23" t="n"/>
-      <c r="R9" s="24">
+      <c r="Q9" s="21" t="n"/>
+      <c r="R9" s="22">
         <f>+R7-R8</f>
         <v/>
       </c>
-      <c r="S9" s="23" t="n"/>
-      <c r="T9" s="24">
+      <c r="S9" s="21" t="n"/>
+      <c r="T9" s="22">
         <f>+T7-T8</f>
         <v/>
       </c>
-      <c r="U9" s="25" t="n"/>
-    </row>
-    <row r="10" ht="15" customHeight="1" thickTop="1">
-      <c r="A10" s="26" t="n"/>
-      <c r="B10" s="26" t="n">
+      <c r="U9" s="23" t="n"/>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="69" thickTop="1">
+      <c r="A10" s="24" t="n"/>
+      <c r="B10" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="26" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="27" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="27" t="n"/>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="27" t="n"/>
-      <c r="K10" s="4" t="n"/>
-      <c r="L10" s="8" t="n"/>
-      <c r="M10" s="4" t="n"/>
-      <c r="N10" s="27" t="n"/>
-      <c r="O10" s="27" t="n"/>
-      <c r="P10" s="27" t="n"/>
-      <c r="Q10" s="27" t="n"/>
-      <c r="R10" s="27" t="n"/>
-      <c r="S10" s="4" t="n"/>
-      <c r="T10" s="27" t="n"/>
-      <c r="U10" s="4" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+      <c r="F10" s="25" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="2" t="n"/>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="6" t="n"/>
+      <c r="M10" s="2" t="n"/>
+      <c r="N10" s="25" t="n"/>
+      <c r="O10" s="25" t="n"/>
+      <c r="P10" s="25" t="n"/>
+      <c r="Q10" s="25" t="n"/>
+      <c r="R10" s="25" t="n"/>
+      <c r="S10" s="2" t="n"/>
+      <c r="T10" s="25" t="n"/>
+      <c r="U10" s="2" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>sales value diff</t>
         </is>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="27">
         <f>+D7-F8-H8-L8-J8-R8-T8-N8-P8</f>
         <v/>
       </c>
-      <c r="F11" s="30" t="n"/>
-      <c r="M11" s="30" t="n"/>
+      <c r="F11" s="72" t="n"/>
+      <c r="M11" s="72" t="n"/>
     </row>
     <row r="12">
-      <c r="F12" s="30" t="n"/>
-      <c r="G12" s="30" t="n"/>
-      <c r="H12" s="31" t="inlineStr">
+      <c r="F12" s="72" t="n"/>
+      <c r="G12" s="72" t="n"/>
+      <c r="H12" s="29" t="inlineStr">
         <is>
           <t>Petrol</t>
         </is>
       </c>
-      <c r="I12" s="31" t="inlineStr">
+      <c r="I12" s="29" t="inlineStr">
         <is>
           <t>Diesal</t>
         </is>
       </c>
-      <c r="J12" s="31" t="inlineStr">
+      <c r="J12" s="29" t="inlineStr">
         <is>
           <t>Power</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="59" t="inlineStr">
+      <c r="A13" s="58" t="inlineStr">
         <is>
           <t>CREDIT DETAIL</t>
         </is>
       </c>
-      <c r="B13" s="74" t="n"/>
-      <c r="C13" s="74" t="n"/>
-      <c r="D13" s="74" t="n"/>
-      <c r="E13" s="74" t="n"/>
-      <c r="F13" s="66" t="n"/>
-      <c r="H13" s="32" t="n"/>
-      <c r="I13" s="41" t="n"/>
-      <c r="J13" s="32" t="n"/>
-      <c r="P13" t="n">
-        <v>31124</v>
-      </c>
+      <c r="B13" s="59" t="n"/>
+      <c r="C13" s="59" t="n"/>
+      <c r="D13" s="59" t="n"/>
+      <c r="E13" s="59" t="n"/>
+      <c r="F13" s="57" t="n"/>
+      <c r="H13" s="79" t="n"/>
+      <c r="I13" s="80" t="n"/>
+      <c r="J13" s="79" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>particular</t>
         </is>
       </c>
-      <c r="B14" s="31" t="inlineStr">
+      <c r="B14" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">Type </t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="D14" s="33" t="inlineStr">
+      <c r="D14" s="31" t="inlineStr">
         <is>
           <t>RATE</t>
         </is>
       </c>
-      <c r="E14" s="33" t="inlineStr">
+      <c r="E14" s="31" t="inlineStr">
         <is>
           <t>AMOUNT</t>
         </is>
       </c>
-      <c r="F14" s="34" t="inlineStr">
+      <c r="F14" s="32" t="inlineStr">
         <is>
           <t>inv no</t>
         </is>
       </c>
-      <c r="H14" s="32" t="n"/>
-      <c r="I14" s="41" t="n"/>
-      <c r="J14" s="32" t="n"/>
-      <c r="K14" s="35" t="inlineStr">
-        <is>
-          <t>Amount</t>
-        </is>
-      </c>
-      <c r="L14" s="36" t="n"/>
-      <c r="M14" s="36" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="P14" t="n">
-        <v>16868.8</v>
-      </c>
+      <c r="H14" s="79" t="n"/>
+      <c r="I14" s="80" t="n"/>
+      <c r="J14" s="79" t="n"/>
+      <c r="K14" s="74" t="n"/>
+      <c r="L14" s="74" t="n"/>
+      <c r="M14" s="74" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="37" t="n"/>
-      <c r="B15" s="38" t="inlineStr">
+      <c r="A15" s="33" t="n"/>
+      <c r="B15" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="29">
         <f>+E15/D15</f>
         <v/>
       </c>
-      <c r="D15" s="32">
+      <c r="D15" s="79">
         <f>+VLOOKUP(B15,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E15" s="75" t="n"/>
-      <c r="F15" s="38" t="n"/>
-      <c r="H15" s="41" t="n"/>
-      <c r="I15" s="41" t="n"/>
-      <c r="J15" s="41" t="n"/>
-      <c r="K15" s="42" t="n"/>
-      <c r="L15" s="32">
-        <f>+C4</f>
-        <v/>
-      </c>
-      <c r="M15" s="32">
-        <f>+K15/L15</f>
-        <v/>
-      </c>
-      <c r="P15" t="n">
-        <v>38634.78</v>
-      </c>
-      <c r="V15">
-        <f>2123+9236+3417.23+18069.1</f>
-        <v/>
-      </c>
+      <c r="E15" s="81" t="n"/>
+      <c r="F15" s="34" t="n"/>
+      <c r="H15" s="80" t="n"/>
+      <c r="I15" s="80" t="n"/>
+      <c r="J15" s="80" t="n"/>
+      <c r="K15" s="72" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="37" t="n"/>
-      <c r="B16" s="38" t="inlineStr">
+      <c r="A16" s="33" t="n"/>
+      <c r="B16" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="29">
         <f>+E16/D16</f>
         <v/>
       </c>
-      <c r="D16" s="32">
+      <c r="D16" s="79">
         <f>+VLOOKUP(B16,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E16" s="75" t="n"/>
-      <c r="F16" s="38" t="n"/>
-      <c r="H16" s="32">
+      <c r="E16" s="81" t="n"/>
+      <c r="F16" s="34" t="n"/>
+      <c r="H16" s="79">
         <f>+H24/C4</f>
         <v/>
       </c>
-      <c r="I16" s="76">
+      <c r="I16" s="43">
         <f>+I24/C5</f>
         <v/>
       </c>
-      <c r="J16" s="76">
+      <c r="J16" s="43">
         <f>+J24/C6</f>
         <v/>
       </c>
-      <c r="K16" s="42" t="n"/>
-      <c r="L16" s="32">
-        <f>+C5</f>
-        <v/>
-      </c>
-      <c r="M16" s="41">
-        <f>+K16/L16</f>
-        <v/>
-      </c>
-      <c r="P16" t="n">
-        <v>68665.22</v>
-      </c>
+      <c r="K16" s="72" t="n"/>
+      <c r="M16" s="72" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="37" t="n"/>
-      <c r="B17" s="38" t="inlineStr">
+      <c r="A17" s="33" t="n"/>
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C17" s="31">
+      <c r="C17" s="29">
         <f>+E17/D17</f>
         <v/>
       </c>
-      <c r="D17" s="32">
+      <c r="D17" s="79">
         <f>+VLOOKUP(B17,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E17" s="77" t="n"/>
-      <c r="F17" s="38" t="n"/>
-      <c r="H17" s="30" t="n"/>
-      <c r="K17" s="41" t="n"/>
-      <c r="L17" s="32">
-        <f>+C4</f>
-        <v/>
-      </c>
-      <c r="M17" s="32">
-        <f>+K17/L17</f>
-        <v/>
-      </c>
-      <c r="P17" t="n">
-        <v>62847.72</v>
-      </c>
+      <c r="E17" s="82" t="n"/>
+      <c r="F17" s="34" t="n"/>
+      <c r="H17" s="72" t="n"/>
+      <c r="K17" s="72" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="37" t="n"/>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="A18" s="33" t="n"/>
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C18" s="31">
+      <c r="C18" s="29">
         <f>+E18/D18</f>
         <v/>
       </c>
-      <c r="D18" s="32">
+      <c r="D18" s="79">
         <f>+VLOOKUP(B18,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E18" s="77" t="n"/>
-      <c r="F18" s="38" t="n"/>
-      <c r="P18" t="n">
-        <v>199</v>
-      </c>
+      <c r="E18" s="82" t="n"/>
+      <c r="F18" s="34" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="37" t="n"/>
-      <c r="B19" s="38" t="inlineStr">
+      <c r="A19" s="33" t="n"/>
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="29">
         <f>+E19/D19</f>
         <v/>
       </c>
-      <c r="D19" s="32">
+      <c r="D19" s="79">
         <f>+VLOOKUP(B19,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E19" s="77" t="n"/>
-      <c r="F19" s="49" t="n"/>
-      <c r="H19">
-        <f>179130.55+24221.9</f>
-        <v/>
-      </c>
-      <c r="K19" s="47" t="n"/>
-      <c r="L19" s="32">
-        <f>+L16</f>
-        <v/>
-      </c>
-      <c r="M19" s="41">
-        <f>+K19/L19</f>
-        <v/>
-      </c>
-      <c r="P19" t="n">
-        <v>163569</v>
-      </c>
+      <c r="E19" s="82" t="n"/>
+      <c r="F19" s="39" t="n"/>
+      <c r="K19" s="72" t="n"/>
+      <c r="M19" s="72" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="37" t="n"/>
-      <c r="B20" s="38" t="inlineStr">
+      <c r="A20" s="33" t="n"/>
+      <c r="B20" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="29">
         <f>+E20/D20</f>
         <v/>
       </c>
-      <c r="D20" s="32">
+      <c r="D20" s="79">
         <f>+VLOOKUP(B20,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E20" s="77" t="n"/>
-      <c r="F20" s="32" t="n"/>
-      <c r="K20" s="41">
-        <f>+M20/L20</f>
-        <v/>
-      </c>
-      <c r="L20" s="32">
-        <f>+C4</f>
-        <v/>
-      </c>
-      <c r="M20" s="44" t="n"/>
-      <c r="P20">
-        <f>SUM(P13:P19)</f>
-        <v/>
-      </c>
+      <c r="E20" s="82" t="n"/>
+      <c r="F20" s="79" t="n"/>
+      <c r="K20" s="72" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="38" t="inlineStr">
+      <c r="A21" s="33" t="n"/>
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C21" s="31">
+      <c r="C21" s="29">
         <f>+E21/D21</f>
         <v/>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="79">
         <f>+VLOOKUP(B21,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E21" s="77" t="n"/>
-      <c r="F21" s="40" t="n"/>
-      <c r="H21" s="45" t="n"/>
-      <c r="K21" s="30">
-        <f>+N8-K15</f>
-        <v/>
-      </c>
-      <c r="L21" s="32">
-        <f>+L16</f>
-        <v/>
-      </c>
-      <c r="M21" s="41">
-        <f>+K21/L21</f>
-        <v/>
-      </c>
+      <c r="E21" s="82" t="n"/>
+      <c r="F21" s="35" t="n"/>
+      <c r="H21" s="71" t="n"/>
+      <c r="K21" s="72" t="n"/>
+      <c r="M21" s="72" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="37" t="n"/>
-      <c r="B22" s="38" t="inlineStr">
+      <c r="A22" s="33" t="n"/>
+      <c r="B22" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C22" s="31">
+      <c r="C22" s="29">
         <f>+E22/D22</f>
         <v/>
       </c>
-      <c r="D22" s="32">
+      <c r="D22" s="79">
         <f>+VLOOKUP(B22,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E22" s="77" t="n"/>
-      <c r="F22" s="32" t="n"/>
+      <c r="E22" s="82" t="n"/>
+      <c r="F22" s="79" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="38" t="n"/>
-      <c r="B23" s="38" t="inlineStr">
+      <c r="A23" s="34" t="n"/>
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C23" s="31">
+      <c r="C23" s="29">
         <f>+E23/D23</f>
         <v/>
       </c>
-      <c r="D23" s="32">
+      <c r="D23" s="79">
         <f>+VLOOKUP(B23,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E23" s="77" t="n"/>
-      <c r="F23" s="32" t="n"/>
+      <c r="E23" s="82" t="n"/>
+      <c r="F23" s="79" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="38" t="n"/>
-      <c r="B24" s="38" t="inlineStr">
+      <c r="A24" s="34" t="n"/>
+      <c r="B24" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C24" s="31">
+      <c r="C24" s="29">
         <f>+E24/D24</f>
         <v/>
       </c>
-      <c r="D24" s="32">
+      <c r="D24" s="79">
         <f>+VLOOKUP(B24,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E24" s="31" t="n"/>
-      <c r="F24" s="32" t="n"/>
-      <c r="H24" s="30">
-        <f>+H13+H14+H15</f>
-        <v/>
-      </c>
-      <c r="I24" s="30">
-        <f>+I13+I14+I15</f>
-        <v/>
-      </c>
-      <c r="J24" s="30">
-        <f>+J13+J14+J15</f>
-        <v/>
-      </c>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="79" t="n"/>
+      <c r="H24" s="72" t="n"/>
+      <c r="I24" s="72" t="n"/>
+      <c r="J24" s="72" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="38" t="n"/>
-      <c r="B25" s="38" t="inlineStr">
+      <c r="A25" s="34" t="n"/>
+      <c r="B25" s="34" t="inlineStr">
         <is>
           <t>diesal</t>
         </is>
       </c>
-      <c r="C25" s="31">
+      <c r="C25" s="29">
         <f>+E25/D25</f>
         <v/>
       </c>
-      <c r="D25" s="32">
+      <c r="D25" s="79">
         <f>+VLOOKUP(B25,A$4:C$6,3,0)</f>
         <v/>
       </c>
-      <c r="E25" s="31" t="n"/>
-      <c r="F25" s="32" t="n"/>
-      <c r="H25" s="30" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="79" t="n"/>
+      <c r="H25" s="72" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="n"/>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="31">
+      <c r="A26" s="79" t="n"/>
+      <c r="B26" s="79" t="n"/>
+      <c r="C26" s="29">
         <f>SUM(C15:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="31" t="n"/>
-      <c r="E26" s="31">
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29">
         <f>SUM(E15:E25)</f>
         <v/>
       </c>
-      <c r="F26" s="32" t="n"/>
-      <c r="N26" t="n">
-        <v>1</v>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>Unlimited power by Anthony robbins</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="H27">
-        <f>1037.67*108.45</f>
-        <v/>
-      </c>
-      <c r="N27" t="n">
-        <v>2</v>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>Compund effect</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>by darren hardy</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="N28" t="n">
-        <v>3</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>leaders eat last</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="N29" t="n">
-        <v>4</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>attitute is everything</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>jef caller</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="N30" t="n">
-        <v>5</v>
-      </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>seven strategies</t>
-        </is>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>by jim rohn</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="C32">
-        <f>+C15+C16</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>gdfg</t>
-        </is>
-      </c>
-    </row>
+      <c r="F26" s="79" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
     <row r="50">
       <c r="E50" t="n">
         <v>9</v>
@@ -2111,82 +1919,11 @@
     <mergeCell ref="U2:U3"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="D2:D3"/>
+    <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="A8:B8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A3:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
-  <cols>
-    <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="17.88671875" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="17.5546875" customWidth="1" min="4" max="4"/>
-    <col width="22.6640625" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="11.109375" bestFit="1" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="3">
-      <c r="A3" s="59" t="inlineStr">
-        <is>
-          <t>CREDIT DETAIL</t>
-        </is>
-      </c>
-      <c r="B3" s="74" t="n"/>
-      <c r="C3" s="74" t="n"/>
-      <c r="D3" s="74" t="n"/>
-      <c r="E3" s="74" t="n"/>
-      <c r="F3" s="74" t="n"/>
-      <c r="G3" s="66" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="32" t="n"/>
-      <c r="B4" s="31" t="inlineStr">
-        <is>
-          <t>particular</t>
-        </is>
-      </c>
-      <c r="C4" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type </t>
-        </is>
-      </c>
-      <c r="D4" s="33" t="inlineStr">
-        <is>
-          <t>QTY</t>
-        </is>
-      </c>
-      <c r="E4" s="33" t="inlineStr">
-        <is>
-          <t>RATE</t>
-        </is>
-      </c>
-      <c r="F4" s="33" t="inlineStr">
-        <is>
-          <t>AMOUNT</t>
-        </is>
-      </c>
-      <c r="G4" s="34" t="inlineStr">
-        <is>
-          <t>inv no</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A3:G3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>